<commit_message>
Upload Center workbook: rebuilt so its Kind drop-down has Plant Managers
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GaDSmfMAZUyAwfZW2Bv1Mz
</commit_message>
<xml_diff>
--- a/public/templates/Plant-Setup-Workbook.xlsx
+++ b/public/templates/Plant-Setup-Workbook.xlsx
@@ -4833,7 +4833,7 @@
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>The station kinds on Station Codes. Choices: Case Loadout, Case Unloading, Tote Loadout, Boxing Loadout, Yard Services, Garage, Driver Room Check-In Station, Driver's Kiosk Station.</t>
+          <t>The station kinds on Station Codes. Choices: Case Loadout, Case Unloading, Tote Loadout, Boxing Loadout, Yard Services, Garage, Driver Room Check-In Station, Driver's Kiosk Station, Plant Managers.</t>
         </is>
       </c>
       <c r="F153" s="4" t="inlineStr">
@@ -6101,8 +6101,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B3001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Pick one of: Case Loadout, Case Unloading, Tote Loadout, Boxing Loadout, Yard Services, Garage, Driver Room Check-In Station, Driver's Kiosk Station" type="list" errorStyle="stop">
-      <formula1>"Case Loadout,Case Unloading,Tote Loadout,Boxing Loadout,Yard Services,Garage,Driver Room Check-In Station,Driver's Kiosk Station"</formula1>
+    <dataValidation sqref="B2:B3001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Pick one of: Case Loadout, Case Unloading, Tote Loadout, Boxing Loadout, Yard Services, Garage, Driver Room Check-In Station, Driver's Kiosk Station, Plant Managers" type="list" errorStyle="stop">
+      <formula1>"Case Loadout,Case Unloading,Tote Loadout,Boxing Loadout,Yard Services,Garage,Driver Room Check-In Station,Driver's Kiosk Station,Plant Managers"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>